<commit_message>
Stage 8 fixes: C-018
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Client_Work/QP07/MV-2018-336/MV-2018-336_AssayWorksheet_022819_v03.xlsx
+++ b/output/archive/MerrivossData/Client_Work/QP07/MV-2018-336/MV-2018-336_AssayWorksheet_022819_v03.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -751,6 +751,31 @@
       <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Helen Marchwood, 02/28/2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>The soluble-branch decision rests on interpretable soluble compounds such as QP07-08608 and QP07-08648 after run acceptance. Recovery- or solubility-limited rows do not independently establish efflux liability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Accession-lot source</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>M18/BIO/07750: compound-linked analyte cards hold the received lot, assay aliquot and matrix/insert links for every compound in the assay tables.</t>
         </is>
       </c>
     </row>
@@ -769,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -789,7 +814,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>10 µM dosing, pH 7.4, 120 min at 37 °C. Efflux ratio is Papp B-A over Papp A-B; ratios above 2.5 were carried into the redesign discussion.</t>
+          <t>10 µM dosing, pH 7.4, 120 min at 37 °C. Efflux ratio is Papp B-A over Papp A-B. Run acceptance requires monolayer integrity before/after exposure, paracellular-marker, reference-flux and vehicle controls against study-plan limits; the insert-linked acceptance and compound accession-lot records are retained under M18/BIO/07750. Accepted controls do not remove compound-specific recovery or solubility limitations.</t>
         </is>
       </c>
     </row>
@@ -1427,6 +1452,56 @@
       </c>
       <c r="E36" s="5" t="n">
         <v>90</v>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Qualified rows</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Recovery below the study-plan window: QP07-08500, QP07-08524, QP07-08542, QP07-08600, QP07-08614, QP07-08638, QP07-08650 and QP07-08674. Retain observed flux values as qualified; exclude from the unqualified soluble-branch comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Solubility limitation</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Nominal dosing exceeds measured kinetic solubility for QP07-08522, QP07-08542, QP07-08584, QP07-08600, QP07-08618, QP07-08642 and QP07-08684. Apparent permeability/ratios are qualified and do not establish intrinsic efflux; no replacement measurements are inferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Interpretable soluble branch</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>QP07-08608 and QP07-08648 have soluble dosing conditions, adequate reported recovery and elevated efflux ratios. These support the exposed-amine redesign after matrix acceptance, without relying on qualified rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Source linkage</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>M18/BIO/07750: each table compound maps by its identifier to its analyte card, received accession lot, assay aliquot and insert-linked acceptance record.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1463,7 +1538,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>RED device, 4 h at 37 °C, buffer against plasma. Recovery on both chambers reported; the run sheet notes any recovery under 80%.</t>
+          <t>RED device, 4 h at 37 °C, buffer against plasma. Total recovery across both chambers is reported as Recovery (%). The run sheet notes any recovery under 80%.</t>
         </is>
       </c>
     </row>

</xml_diff>